<commit_message>
Replace two revised sensory workbooks and add audit summary
</commit_message>
<xml_diff>
--- a/英文/单体混合感官特征理化数据.xlsx
+++ b/英文/单体混合感官特征理化数据.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\教学及研究生培养\毕业设计\2025届本科毕业作业老师报题相关附件\毕业论文\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\24252\Desktop\PPT\课题\26年\26.10\英文\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC0A1CA-D833-4145-8D27-89C3DA05E363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DCE4695-F3E7-4543-B387-CC75CD02497B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{A40A38D2-C497-4439-9AEB-F5807B99F314}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="22308" windowHeight="13176" activeTab="1" xr2:uid="{A40A38D2-C497-4439-9AEB-F5807B99F314}"/>
   </bookViews>
   <sheets>
     <sheet name="组合数据" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="444">
   <si>
     <t>Sample</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -5908,6 +5907,72 @@
       </rPr>
       <t/>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>丁酸</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(C1)</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>丁酸</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(C6)</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="1"/>
+        <charset val="134"/>
+      </rPr>
+      <t>异丁酸乙酯（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>C8)</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -6532,39 +6597,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2818894E-F368-4508-A891-42EE1AB06FE7}">
   <dimension ref="A1:AQ157"/>
-  <sheetFormatPr defaultColWidth="8.1640625" defaultRowHeight="15.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.1640625" style="25"/>
-    <col min="2" max="2" width="21.58203125" style="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.109375" style="25"/>
+    <col min="2" max="2" width="21.5546875" style="23" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="9.4140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" style="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.44140625" style="24" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.5" style="24" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="24" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5" style="24" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.25" style="24" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.83203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.21875" style="24" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.77734375" style="24" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.5" style="24" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.4140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.44140625" style="24" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.75" style="24" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.4140625" style="24" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.4140625" style="24" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.83203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.58203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.83203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.25" style="24" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.58203125" style="24" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.5" style="25" bestFit="1" customWidth="1"/>
-    <col min="29" max="41" width="8.1640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.83203125" style="25" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.1640625" style="25" bestFit="1" customWidth="1"/>
-    <col min="44" max="16384" width="8.1640625" style="25"/>
+    <col min="20" max="20" width="19.77734375" style="24" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.77734375" style="24" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.5546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.77734375" style="24" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.21875" style="24" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.5546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.44140625" style="25" bestFit="1" customWidth="1"/>
+    <col min="29" max="41" width="8.109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.77734375" style="25" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="44" max="16384" width="8.109375" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A1" s="31" t="s">
         <v>349</v>
       </c>
@@ -6695,7 +6760,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
         <v>350</v>
       </c>
@@ -6754,7 +6819,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" s="32" t="s">
         <v>351</v>
       </c>
@@ -6813,7 +6878,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
         <v>352</v>
       </c>
@@ -6872,7 +6937,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" s="32" t="s">
         <v>353</v>
       </c>
@@ -6931,7 +6996,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" s="32" t="s">
         <v>354</v>
       </c>
@@ -6990,7 +7055,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" s="32" t="s">
         <v>355</v>
       </c>
@@ -7049,7 +7114,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" s="32" t="s">
         <v>356</v>
       </c>
@@ -7108,7 +7173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" s="32" t="s">
         <v>357</v>
       </c>
@@ -7167,7 +7232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" s="32" t="s">
         <v>358</v>
       </c>
@@ -7226,7 +7291,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" s="32" t="s">
         <v>359</v>
       </c>
@@ -7285,7 +7350,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" s="32" t="s">
         <v>360</v>
       </c>
@@ -7344,7 +7409,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" s="32" t="s">
         <v>361</v>
       </c>
@@ -7403,7 +7468,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" s="32" t="s">
         <v>362</v>
       </c>
@@ -7462,7 +7527,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" s="32" t="s">
         <v>363</v>
       </c>
@@ -7521,7 +7586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" s="32" t="s">
         <v>364</v>
       </c>
@@ -7580,7 +7645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A17" s="32" t="s">
         <v>365</v>
       </c>
@@ -7639,7 +7704,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A18" s="32" t="s">
         <v>366</v>
       </c>
@@ -7698,7 +7763,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A19" s="32" t="s">
         <v>367</v>
       </c>
@@ -7757,7 +7822,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A20" s="32" t="s">
         <v>368</v>
       </c>
@@ -7816,7 +7881,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="21" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A21" s="32" t="s">
         <v>369</v>
       </c>
@@ -7875,7 +7940,7 @@
         <v>0.22222222222222221</v>
       </c>
     </row>
-    <row r="22" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A22" s="32" t="s">
         <v>370</v>
       </c>
@@ -7934,7 +7999,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A23" s="32" t="s">
         <v>371</v>
       </c>
@@ -7993,7 +8058,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A24" s="32" t="s">
         <v>372</v>
       </c>
@@ -8052,7 +8117,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="25" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A25" s="32" t="s">
         <v>373</v>
       </c>
@@ -8111,7 +8176,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="26" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A26" s="32" t="s">
         <v>374</v>
       </c>
@@ -8170,7 +8235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A27" s="32" t="s">
         <v>375</v>
       </c>
@@ -8229,7 +8294,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="28" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A28" s="32" t="s">
         <v>376</v>
       </c>
@@ -8288,7 +8353,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A29" s="32" t="s">
         <v>377</v>
       </c>
@@ -8347,7 +8412,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="30" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A30" s="32" t="s">
         <v>378</v>
       </c>
@@ -8406,7 +8471,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="31" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A31" s="32" t="s">
         <v>379</v>
       </c>
@@ -8465,7 +8530,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="32" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A32" s="32" t="s">
         <v>380</v>
       </c>
@@ -8524,7 +8589,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="33" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A33" s="32" t="s">
         <v>381</v>
       </c>
@@ -8583,7 +8648,7 @@
         <v>0.27777777777777779</v>
       </c>
     </row>
-    <row r="34" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A34" s="32" t="s">
         <v>382</v>
       </c>
@@ -8642,7 +8707,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="35" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A35" s="32" t="s">
         <v>383</v>
       </c>
@@ -8701,7 +8766,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="36" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A36" s="32" t="s">
         <v>384</v>
       </c>
@@ -8760,7 +8825,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A37" s="32" t="s">
         <v>385</v>
       </c>
@@ -8819,7 +8884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A38" s="32" t="s">
         <v>386</v>
       </c>
@@ -8878,7 +8943,7 @@
         <v>0.27777777777777779</v>
       </c>
     </row>
-    <row r="39" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A39" s="32" t="s">
         <v>387</v>
       </c>
@@ -8937,7 +9002,7 @@
         <v>0.22222222222222221</v>
       </c>
     </row>
-    <row r="40" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A40" s="32" t="s">
         <v>388</v>
       </c>
@@ -8996,7 +9061,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="41" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A41" s="32" t="s">
         <v>389</v>
       </c>
@@ -9055,7 +9120,7 @@
         <v>0.22222222222222221</v>
       </c>
     </row>
-    <row r="42" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A42" s="32" t="s">
         <v>390</v>
       </c>
@@ -9114,7 +9179,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="43" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A43" s="32" t="s">
         <v>391</v>
       </c>
@@ -9173,7 +9238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A44" s="32" t="s">
         <v>392</v>
       </c>
@@ -9232,7 +9297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A45" s="32" t="s">
         <v>393</v>
       </c>
@@ -9291,7 +9356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A46" s="32" t="s">
         <v>394</v>
       </c>
@@ -9350,7 +9415,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="47" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A47" s="32" t="s">
         <v>395</v>
       </c>
@@ -9409,7 +9474,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A48" s="32" t="s">
         <v>396</v>
       </c>
@@ -9468,7 +9533,7 @@
         <v>0.22222222222222221</v>
       </c>
     </row>
-    <row r="49" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A49" s="32" t="s">
         <v>397</v>
       </c>
@@ -9527,7 +9592,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A50" s="32" t="s">
         <v>398</v>
       </c>
@@ -9586,7 +9651,7 @@
         <v>0.27777777777777779</v>
       </c>
     </row>
-    <row r="51" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A51" s="32" t="s">
         <v>399</v>
       </c>
@@ -9645,7 +9710,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="52" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A52" s="32" t="s">
         <v>400</v>
       </c>
@@ -9704,7 +9769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A53" s="32" t="s">
         <v>401</v>
       </c>
@@ -9763,7 +9828,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="54" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A54" s="32" t="s">
         <v>402</v>
       </c>
@@ -9822,7 +9887,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="55" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A55" s="32" t="s">
         <v>403</v>
       </c>
@@ -9881,7 +9946,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="56" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A56" s="32" t="s">
         <v>404</v>
       </c>
@@ -9940,7 +10005,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A57" s="32" t="s">
         <v>405</v>
       </c>
@@ -9999,7 +10064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A58" s="32" t="s">
         <v>406</v>
       </c>
@@ -10058,7 +10123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A59" s="32" t="s">
         <v>407</v>
       </c>
@@ -10117,7 +10182,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A60" s="32" t="s">
         <v>408</v>
       </c>
@@ -10176,7 +10241,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A61" s="32" t="s">
         <v>409</v>
       </c>
@@ -10235,7 +10300,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="62" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A62" s="32" t="s">
         <v>410</v>
       </c>
@@ -10294,7 +10359,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="63" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A63" s="32" t="s">
         <v>411</v>
       </c>
@@ -10353,7 +10418,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="64" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A64" s="32" t="s">
         <v>412</v>
       </c>
@@ -10412,7 +10477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A65" s="32" t="s">
         <v>413</v>
       </c>
@@ -10471,7 +10536,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A66" s="32" t="s">
         <v>414</v>
       </c>
@@ -10530,7 +10595,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="67" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A67" s="32" t="s">
         <v>415</v>
       </c>
@@ -10589,7 +10654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A68" s="32" t="s">
         <v>416</v>
       </c>
@@ -10648,7 +10713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A69" s="32" t="s">
         <v>417</v>
       </c>
@@ -10707,7 +10772,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A70" s="32" t="s">
         <v>418</v>
       </c>
@@ -10766,7 +10831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A71" s="32" t="s">
         <v>419</v>
       </c>
@@ -10825,7 +10890,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A72" s="32" t="s">
         <v>420</v>
       </c>
@@ -10884,7 +10949,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A73" s="32" t="s">
         <v>421</v>
       </c>
@@ -10943,7 +11008,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="74" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A74" s="32" t="s">
         <v>422</v>
       </c>
@@ -11002,7 +11067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A75" s="32" t="s">
         <v>423</v>
       </c>
@@ -11061,7 +11126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A76" s="32" t="s">
         <v>424</v>
       </c>
@@ -11120,7 +11185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A77" s="32" t="s">
         <v>425</v>
       </c>
@@ -11179,7 +11244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A78" s="32" t="s">
         <v>426</v>
       </c>
@@ -11238,7 +11303,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="79" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A79" s="32" t="s">
         <v>427</v>
       </c>
@@ -11297,7 +11362,7 @@
         <v>0.22222222222222221</v>
       </c>
     </row>
-    <row r="80" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A80" s="32" t="s">
         <v>428</v>
       </c>
@@ -11356,7 +11421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A81" s="32" t="s">
         <v>429</v>
       </c>
@@ -11415,7 +11480,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="82" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A82" s="32" t="s">
         <v>430</v>
       </c>
@@ -11474,7 +11539,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A83" s="32" t="s">
         <v>431</v>
       </c>
@@ -11533,7 +11598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A84" s="32" t="s">
         <v>432</v>
       </c>
@@ -11592,7 +11657,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="85" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A85" s="32" t="s">
         <v>433</v>
       </c>
@@ -11651,7 +11716,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="86" spans="1:43" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A86" s="32" t="s">
         <v>434</v>
       </c>
@@ -11710,7 +11775,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="87" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A87" s="32" t="s">
         <v>435</v>
       </c>
@@ -11769,7 +11834,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="88" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A88" s="32" t="s">
         <v>436</v>
       </c>
@@ -11828,7 +11893,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="89" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A89" s="32" t="s">
         <v>437</v>
       </c>
@@ -11887,7 +11952,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A90" s="32" t="s">
         <v>438</v>
       </c>
@@ -11946,7 +12011,7 @@
         <v>0.22222222222222221</v>
       </c>
     </row>
-    <row r="91" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A91" s="32" t="s">
         <v>439</v>
       </c>
@@ -12005,7 +12070,7 @@
         <v>5.5555555555555552E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A92" s="32" t="s">
         <v>440</v>
       </c>
@@ -12064,7 +12129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A93" s="29" t="s">
         <v>267</v>
       </c>
@@ -12192,7 +12257,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="94" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A94" s="29" t="s">
         <v>92</v>
       </c>
@@ -12320,7 +12385,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A95" s="29" t="s">
         <v>93</v>
       </c>
@@ -12451,7 +12516,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A96" s="29" t="s">
         <v>94</v>
       </c>
@@ -12579,7 +12644,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="97" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A97" s="29" t="s">
         <v>95</v>
       </c>
@@ -12707,7 +12772,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A98" s="29" t="s">
         <v>96</v>
       </c>
@@ -12835,7 +12900,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A99" s="29" t="s">
         <v>97</v>
       </c>
@@ -12963,7 +13028,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="100" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A100" s="29" t="s">
         <v>98</v>
       </c>
@@ -13091,7 +13156,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="101" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A101" s="29" t="s">
         <v>99</v>
       </c>
@@ -13219,7 +13284,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A102" s="29" t="s">
         <v>100</v>
       </c>
@@ -13347,7 +13412,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="103" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A103" s="29" t="s">
         <v>101</v>
       </c>
@@ -13475,7 +13540,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="104" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A104" s="29" t="s">
         <v>102</v>
       </c>
@@ -13603,7 +13668,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="105" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A105" s="29" t="s">
         <v>103</v>
       </c>
@@ -13731,7 +13796,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="106" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A106" s="29" t="s">
         <v>104</v>
       </c>
@@ -13859,7 +13924,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="107" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A107" s="29" t="s">
         <v>105</v>
       </c>
@@ -13987,7 +14052,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="108" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A108" s="29" t="s">
         <v>106</v>
       </c>
@@ -14115,7 +14180,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="109" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A109" s="29" t="s">
         <v>107</v>
       </c>
@@ -14243,7 +14308,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="110" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A110" s="29" t="s">
         <v>108</v>
       </c>
@@ -14371,7 +14436,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="111" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A111" s="29" t="s">
         <v>109</v>
       </c>
@@ -14499,7 +14564,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="112" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A112" s="29" t="s">
         <v>110</v>
       </c>
@@ -14627,7 +14692,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="113" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A113" s="29" t="s">
         <v>111</v>
       </c>
@@ -14755,7 +14820,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="114" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A114" s="29" t="s">
         <v>112</v>
       </c>
@@ -14886,7 +14951,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A115" s="29" t="s">
         <v>113</v>
       </c>
@@ -15014,7 +15079,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="116" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A116" s="29" t="s">
         <v>114</v>
       </c>
@@ -15145,7 +15210,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A117" s="29" t="s">
         <v>115</v>
       </c>
@@ -15273,7 +15338,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="118" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A118" s="29" t="s">
         <v>116</v>
       </c>
@@ -15401,7 +15466,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="119" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A119" s="29" t="s">
         <v>117</v>
       </c>
@@ -15529,7 +15594,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="120" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A120" s="29" t="s">
         <v>118</v>
       </c>
@@ -15657,7 +15722,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A121" s="29" t="s">
         <v>119</v>
       </c>
@@ -15785,7 +15850,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="122" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A122" s="29" t="s">
         <v>120</v>
       </c>
@@ -15913,7 +15978,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="123" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A123" s="29" t="s">
         <v>121</v>
       </c>
@@ -16044,7 +16109,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A124" s="29" t="s">
         <v>122</v>
       </c>
@@ -16172,7 +16237,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="125" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A125" s="29" t="s">
         <v>123</v>
       </c>
@@ -16300,7 +16365,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="126" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A126" s="29" t="s">
         <v>124</v>
       </c>
@@ -16428,7 +16493,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A127" s="29" t="s">
         <v>125</v>
       </c>
@@ -16556,7 +16621,7 @@
         <v>0.313</v>
       </c>
     </row>
-    <row r="128" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A128" s="29" t="s">
         <v>126</v>
       </c>
@@ -16684,7 +16749,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="129" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A129" s="29" t="s">
         <v>127</v>
       </c>
@@ -16812,7 +16877,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="130" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A130" s="29" t="s">
         <v>128</v>
       </c>
@@ -16940,7 +17005,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="131" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A131" s="29" t="s">
         <v>129</v>
       </c>
@@ -17068,7 +17133,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="132" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A132" s="29" t="s">
         <v>130</v>
       </c>
@@ -17196,7 +17261,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="133" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A133" s="29" t="s">
         <v>131</v>
       </c>
@@ -17324,7 +17389,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="134" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A134" s="29" t="s">
         <v>132</v>
       </c>
@@ -17452,7 +17517,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="135" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A135" s="29" t="s">
         <v>133</v>
       </c>
@@ -17580,7 +17645,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="136" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A136" s="29" t="s">
         <v>134</v>
       </c>
@@ -17708,7 +17773,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="137" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A137" s="29" t="s">
         <v>135</v>
       </c>
@@ -17836,7 +17901,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="138" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A138" s="29" t="s">
         <v>136</v>
       </c>
@@ -17964,7 +18029,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="139" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A139" s="29" t="s">
         <v>137</v>
       </c>
@@ -18092,7 +18157,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="140" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A140" s="29" t="s">
         <v>138</v>
       </c>
@@ -18220,7 +18285,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="141" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A141" s="29" t="s">
         <v>139</v>
       </c>
@@ -18351,7 +18416,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A142" s="29" t="s">
         <v>140</v>
       </c>
@@ -18479,7 +18544,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="143" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A143" s="29" t="s">
         <v>141</v>
       </c>
@@ -18607,7 +18672,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="144" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A144" s="29" t="s">
         <v>142</v>
       </c>
@@ -18735,7 +18800,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="145" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A145" s="29" t="s">
         <v>143</v>
       </c>
@@ -18863,7 +18928,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="146" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A146" s="29" t="s">
         <v>144</v>
       </c>
@@ -18991,7 +19056,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="147" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A147" s="29" t="s">
         <v>145</v>
       </c>
@@ -19119,7 +19184,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="148" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A148" s="29" t="s">
         <v>146</v>
       </c>
@@ -19247,7 +19312,7 @@
         <v>0.188</v>
       </c>
     </row>
-    <row r="149" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A149" s="29" t="s">
         <v>147</v>
       </c>
@@ -19375,7 +19440,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="150" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A150" s="29" t="s">
         <v>148</v>
       </c>
@@ -19503,7 +19568,7 @@
         <v>0.27800000000000002</v>
       </c>
     </row>
-    <row r="151" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A151" s="29" t="s">
         <v>149</v>
       </c>
@@ -19631,7 +19696,7 @@
         <v>0.29399999999999998</v>
       </c>
     </row>
-    <row r="152" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A152" s="29" t="s">
         <v>150</v>
       </c>
@@ -19759,7 +19824,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="153" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A153" s="29" t="s">
         <v>151</v>
       </c>
@@ -19887,7 +19952,7 @@
         <v>0.16700000000000001</v>
       </c>
     </row>
-    <row r="154" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A154" s="29" t="s">
         <v>152</v>
       </c>
@@ -20015,7 +20080,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="155" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A155" s="29" t="s">
         <v>153</v>
       </c>
@@ -20143,7 +20208,7 @@
         <v>0.111</v>
       </c>
     </row>
-    <row r="156" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A156" s="29" t="s">
         <v>154</v>
       </c>
@@ -20271,7 +20336,7 @@
         <v>0.11799999999999999</v>
       </c>
     </row>
-    <row r="157" spans="1:42" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A157" s="29" t="s">
         <v>155</v>
       </c>
@@ -20411,14 +20476,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FB4223-8003-4D39-B146-611C375CCF2B}">
-  <dimension ref="A1:B92"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B95"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" style="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20426,7 +20491,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -20434,7 +20499,7 @@
         <v>1.99911833333333</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>23</v>
       </c>
@@ -20442,7 +20507,7 @@
         <v>19.9911833333333</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>38</v>
       </c>
@@ -20450,7 +20515,7 @@
         <v>199.91183333333302</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>53</v>
       </c>
@@ -20458,7 +20523,7 @@
         <v>1999.1183333333299</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>68</v>
       </c>
@@ -20466,7 +20531,7 @@
         <v>19991.183333333302</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>80</v>
       </c>
@@ -20474,7 +20539,7 @@
         <v>199911.83333333299</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
@@ -20482,7 +20547,7 @@
         <v>39.999085333333305</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>27</v>
       </c>
@@ -20490,7 +20555,7 @@
         <v>399.99085333333301</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>42</v>
       </c>
@@ -20498,7 +20563,7 @@
         <v>3999.9085333333301</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>57</v>
       </c>
@@ -20506,7 +20571,7 @@
         <v>39999.0853333333</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>72</v>
       </c>
@@ -20514,7 +20579,7 @@
         <v>399990.85333333298</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>83</v>
       </c>
@@ -20522,7 +20587,7 @@
         <v>3999908.5333333299</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>14</v>
       </c>
@@ -20530,7 +20595,7 @@
         <v>19999.998991734301</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>29</v>
       </c>
@@ -20538,7 +20603,7 @@
         <v>199999.98991734299</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>44</v>
       </c>
@@ -20546,7 +20611,7 @@
         <v>1999999.8991734302</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>59</v>
       </c>
@@ -20554,7 +20619,7 @@
         <v>19999998.9917343</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>74</v>
       </c>
@@ -20562,7 +20627,7 @@
         <v>199999989.91734299</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>86</v>
       </c>
@@ -20570,7 +20635,7 @@
         <v>249999696.66600001</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>5</v>
       </c>
@@ -20578,7 +20643,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>20</v>
       </c>
@@ -20586,7 +20651,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>35</v>
       </c>
@@ -20594,7 +20659,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>50</v>
       </c>
@@ -20602,7 +20667,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>65</v>
       </c>
@@ -20610,7 +20675,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>77</v>
       </c>
@@ -20618,7 +20683,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>91</v>
       </c>
@@ -20626,537 +20691,561 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="B27" s="15">
+        <v>399.99649333333002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="16">
+      <c r="B28" s="16">
         <v>3999.9964933333299</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="15">
+      <c r="B29" s="15">
         <v>39999.9649333333</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="15">
+      <c r="B30" s="15">
         <v>399999.64933333301</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B31" s="15">
         <v>3999996.4933333299</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="B32" s="15">
+        <v>39999996.493333302</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B33" s="16">
         <v>0.19977033333333299</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+    <row r="34" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B34" s="15">
         <v>1.9977033333333301</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
+    <row r="35" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="15">
+      <c r="B35" s="15">
         <v>19.977033333333299</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="21" t="s">
+    <row r="36" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A36" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B34" s="15">
+      <c r="B36" s="15">
         <v>199.77033333333299</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+    <row r="37" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="15">
+      <c r="B37" s="15">
         <v>1997.70333333333</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B36" s="14">
+      <c r="B38" s="14">
         <v>0.2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B37" s="17">
+      <c r="B39" s="17">
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="14">
+      <c r="B40" s="14">
         <v>20</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B39" s="14">
+      <c r="B41" s="14">
         <v>200</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B40" s="17">
+      <c r="B42" s="17">
         <v>2000</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="22" t="s">
+    <row r="43" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A43" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B41" s="14">
+      <c r="B43" s="14">
         <v>20000</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="21" t="s">
+    <row r="44" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A44" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B42" s="14">
+      <c r="B44" s="14">
         <v>200000</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="6" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="15">
+      <c r="B45" s="15">
         <v>40.000533333333301</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="6" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B44" s="15">
+      <c r="B46" s="15">
         <v>400.005333333333</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="3" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B45" s="15">
+      <c r="B47" s="15">
         <v>4000.0533333333301</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="3" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B46" s="15">
+      <c r="B48" s="15">
         <v>40000.533333333304</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="3" t="s">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="16">
+      <c r="B49" s="16">
         <v>400005.33333333302</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="3" t="s">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B48" s="15">
+      <c r="B50" s="15">
         <v>4000053.3333333302</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="3" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B49" s="17">
+      <c r="B51" s="17">
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="17">
+      <c r="B52" s="17">
         <v>20</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="3" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B51" s="14">
+      <c r="B53" s="14">
         <v>200</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B52" s="14">
+      <c r="B54" s="14">
         <v>2000</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B53" s="14">
+      <c r="B55" s="14">
         <v>20000</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" s="3" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B54" s="14">
+      <c r="B56" s="14">
         <v>200000</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
+    <row r="57" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B55" s="14">
+      <c r="B57" s="14">
         <v>2000000</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" s="3" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B56" s="17">
+      <c r="B58" s="17">
         <v>43.13</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" s="3" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B57" s="17">
+      <c r="B59" s="17">
         <v>431.3</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="6" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B58" s="14">
+      <c r="B60" s="14">
         <v>4313</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="6" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B59" s="14">
+      <c r="B61" s="14">
         <v>43130</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="6" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B60" s="14">
+      <c r="B62" s="14">
         <v>431300</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="6" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="15">
+      <c r="B63" s="15">
         <v>400.00130999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" s="6" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B62" s="16">
+      <c r="B64" s="16">
         <v>4000.0131000000001</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" s="6" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B63" s="15">
+      <c r="B65" s="15">
         <v>40000.131000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="6" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B64" s="16">
+      <c r="B66" s="16">
         <v>400001.31</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="3" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B65" s="15">
+      <c r="B67" s="15">
         <v>4000013.1</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" s="3" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B66" s="15">
+      <c r="B68" s="15">
         <v>40000131</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" s="3" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B67" s="15">
+      <c r="B69" s="15">
         <v>1999.997573333</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="3" t="s">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B68" s="15">
+      <c r="B70" s="15">
         <v>19999.97573333</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" s="3" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B69" s="16">
+      <c r="B71" s="16">
         <v>199999.75733330002</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" s="3" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B70" s="15">
+      <c r="B72" s="15">
         <v>1999997.5733330001</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" s="6" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B71" s="15">
+      <c r="B73" s="15">
         <v>19999975.73333</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="6" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B72" s="15">
+      <c r="B74" s="15">
         <v>199999757.33329999</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="6" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B73" s="14">
+      <c r="B75" s="14">
         <v>40</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="6" t="s">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="17">
+      <c r="B76" s="17">
         <v>400</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" s="6" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B75" s="14">
+      <c r="B77" s="14">
         <v>4000</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="6" t="s">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B76" s="14">
+      <c r="B78" s="14">
         <v>40000</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="3" t="s">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B77" s="17">
+      <c r="B79" s="17">
         <v>400000</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A78" s="3" t="s">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B78" s="14">
+      <c r="B80" s="14">
         <v>4000000</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" s="5" t="s">
+    <row r="81" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A81" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B79" s="14">
+      <c r="B81" s="14">
         <v>40000000</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A80" s="3" t="s">
+    <row r="82" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A82" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="B82" s="14">
+        <v>40000000</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B80" s="15">
+      <c r="B83" s="15">
         <v>3.9998879999999999</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A81" s="3" t="s">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B81" s="15">
+      <c r="B84" s="15">
         <v>39.99888</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A82" s="3" t="s">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B82" s="15">
+      <c r="B85" s="15">
         <v>399.98879999999997</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A83" s="3" t="s">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B83" s="15">
+      <c r="B86" s="15">
         <v>3999.8879999999999</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A84" s="6" t="s">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B84" s="15">
+      <c r="B87" s="15">
         <v>39998.879999999997</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A85" s="6" t="s">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B85" s="15">
+      <c r="B88" s="15">
         <v>399988.80000000005</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A86" s="6" t="s">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B86" s="17">
+      <c r="B89" s="17">
         <v>200</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A87" s="6" t="s">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B87" s="14">
+      <c r="B90" s="14">
         <v>2000</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A88" s="6" t="s">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B88" s="14">
+      <c r="B91" s="14">
         <v>20000</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A89" s="6" t="s">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B89" s="14">
+      <c r="B92" s="14">
         <v>200000</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A90" s="6" t="s">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B90" s="17">
+      <c r="B93" s="17">
         <v>2000000</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A91" s="3" t="s">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B91" s="14">
+      <c r="B94" s="14">
         <v>20000000</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A92" s="4" t="s">
+    <row r="95" spans="1:2" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B92" s="14">
+      <c r="B95" s="14">
         <v>200000000</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B98">
-    <sortCondition ref="A2:A98"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B101">
+    <sortCondition ref="A2:A101"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21166,34 +21255,34 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CFBFCB2-97CB-4AC9-BF07-2E14875400DC}">
   <dimension ref="A1:AA66"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="15.6" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="9.25" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="9.21875" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.58203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.08203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.109375" style="9" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.5" style="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.08203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.44140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.109375" style="9" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="9.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="10.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.08203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="10.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.21875" style="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.109375" style="9" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="14" style="9" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11.33203125" style="9" bestFit="1" customWidth="1"/>
     <col min="27" max="16384" width="8.6640625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="16.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>156</v>
       </c>
@@ -21274,7 +21363,7 @@
       </c>
       <c r="AA1" s="8"/>
     </row>
-    <row r="2" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>181</v>
       </c>
@@ -21355,7 +21444,7 @@
       </c>
       <c r="AA2" s="8"/>
     </row>
-    <row r="3" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>186</v>
       </c>
@@ -21436,7 +21525,7 @@
       </c>
       <c r="AA3" s="8"/>
     </row>
-    <row r="4" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>187</v>
       </c>
@@ -21445,7 +21534,7 @@
       </c>
       <c r="AA4" s="12"/>
     </row>
-    <row r="5" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>188</v>
       </c>
@@ -21478,7 +21567,7 @@
       <c r="Z5" s="19"/>
       <c r="AA5" s="13"/>
     </row>
-    <row r="6" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>189</v>
       </c>
@@ -21511,7 +21600,7 @@
       <c r="Z6" s="20"/>
       <c r="AA6" s="10"/>
     </row>
-    <row r="7" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>190</v>
       </c>
@@ -21544,7 +21633,7 @@
       <c r="Z7" s="10"/>
       <c r="AA7" s="10"/>
     </row>
-    <row r="8" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>191</v>
       </c>
@@ -21577,7 +21666,7 @@
       <c r="Z8" s="10"/>
       <c r="AA8" s="10"/>
     </row>
-    <row r="9" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>192</v>
       </c>
@@ -21610,7 +21699,7 @@
       <c r="Z9" s="10"/>
       <c r="AA9" s="10"/>
     </row>
-    <row r="10" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>193</v>
       </c>
@@ -21645,7 +21734,7 @@
       <c r="Z10" s="10"/>
       <c r="AA10" s="10"/>
     </row>
-    <row r="11" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>194</v>
       </c>
@@ -21680,7 +21769,7 @@
       <c r="Z11" s="10"/>
       <c r="AA11" s="10"/>
     </row>
-    <row r="12" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>195</v>
       </c>
@@ -21715,7 +21804,7 @@
       <c r="Z12" s="10"/>
       <c r="AA12" s="10"/>
     </row>
-    <row r="13" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>196</v>
       </c>
@@ -21750,7 +21839,7 @@
       <c r="Z13" s="10"/>
       <c r="AA13" s="10"/>
     </row>
-    <row r="14" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>197</v>
       </c>
@@ -21785,7 +21874,7 @@
       <c r="Z14" s="10"/>
       <c r="AA14" s="10"/>
     </row>
-    <row r="15" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>198</v>
       </c>
@@ -21820,7 +21909,7 @@
       <c r="Z15" s="10"/>
       <c r="AA15" s="10"/>
     </row>
-    <row r="16" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
         <v>199</v>
       </c>
@@ -21855,7 +21944,7 @@
       <c r="Z16" s="10"/>
       <c r="AA16" s="10"/>
     </row>
-    <row r="17" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
         <v>200</v>
       </c>
@@ -21890,7 +21979,7 @@
       <c r="Z17" s="10"/>
       <c r="AA17" s="10"/>
     </row>
-    <row r="18" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
         <v>201</v>
       </c>
@@ -21925,7 +22014,7 @@
       <c r="Z18" s="10"/>
       <c r="AA18" s="10"/>
     </row>
-    <row r="19" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="11" t="s">
         <v>202</v>
       </c>
@@ -21960,7 +22049,7 @@
       <c r="Z19" s="10"/>
       <c r="AA19" s="10"/>
     </row>
-    <row r="20" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="11" t="s">
         <v>203</v>
       </c>
@@ -21995,7 +22084,7 @@
       <c r="Z20" s="10"/>
       <c r="AA20" s="10"/>
     </row>
-    <row r="21" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="11" t="s">
         <v>204</v>
       </c>
@@ -22030,7 +22119,7 @@
       <c r="Z21" s="10"/>
       <c r="AA21" s="10"/>
     </row>
-    <row r="22" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="11" t="s">
         <v>205</v>
       </c>
@@ -22065,7 +22154,7 @@
       <c r="Z22" s="10"/>
       <c r="AA22" s="10"/>
     </row>
-    <row r="23" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
         <v>206</v>
       </c>
@@ -22100,7 +22189,7 @@
       <c r="Z23" s="10"/>
       <c r="AA23" s="10"/>
     </row>
-    <row r="24" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="11" t="s">
         <v>207</v>
       </c>
@@ -22135,7 +22224,7 @@
       <c r="Z24" s="10"/>
       <c r="AA24" s="10"/>
     </row>
-    <row r="25" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
         <v>208</v>
       </c>
@@ -22172,7 +22261,7 @@
       <c r="Z25" s="10"/>
       <c r="AA25" s="10"/>
     </row>
-    <row r="26" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11" t="s">
         <v>209</v>
       </c>
@@ -22209,7 +22298,7 @@
       <c r="Z26" s="10"/>
       <c r="AA26" s="10"/>
     </row>
-    <row r="27" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11" t="s">
         <v>210</v>
       </c>
@@ -22246,7 +22335,7 @@
       <c r="Z27" s="10"/>
       <c r="AA27" s="10"/>
     </row>
-    <row r="28" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="11" t="s">
         <v>211</v>
       </c>
@@ -22283,7 +22372,7 @@
       <c r="Z28" s="10"/>
       <c r="AA28" s="10"/>
     </row>
-    <row r="29" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="11" t="s">
         <v>212</v>
       </c>
@@ -22320,7 +22409,7 @@
       <c r="Z29" s="10"/>
       <c r="AA29" s="10"/>
     </row>
-    <row r="30" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="11" t="s">
         <v>213</v>
       </c>
@@ -22357,7 +22446,7 @@
       <c r="Z30" s="10"/>
       <c r="AA30" s="10"/>
     </row>
-    <row r="31" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="11" t="s">
         <v>214</v>
       </c>
@@ -22394,7 +22483,7 @@
       <c r="Z31" s="10"/>
       <c r="AA31" s="10"/>
     </row>
-    <row r="32" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="11" t="s">
         <v>215</v>
       </c>
@@ -22431,7 +22520,7 @@
       <c r="Z32" s="10"/>
       <c r="AA32" s="10"/>
     </row>
-    <row r="33" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="11" t="s">
         <v>216</v>
       </c>
@@ -22468,7 +22557,7 @@
       <c r="Z33" s="10"/>
       <c r="AA33" s="10"/>
     </row>
-    <row r="34" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="11" t="s">
         <v>217</v>
       </c>
@@ -22505,7 +22594,7 @@
       <c r="Z34" s="10"/>
       <c r="AA34" s="10"/>
     </row>
-    <row r="35" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="11" t="s">
         <v>218</v>
       </c>
@@ -22542,7 +22631,7 @@
       <c r="Z35" s="10"/>
       <c r="AA35" s="10"/>
     </row>
-    <row r="36" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="11" t="s">
         <v>219</v>
       </c>
@@ -22579,7 +22668,7 @@
       <c r="Z36" s="10"/>
       <c r="AA36" s="10"/>
     </row>
-    <row r="37" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="11" t="s">
         <v>220</v>
       </c>
@@ -22616,7 +22705,7 @@
       <c r="Z37" s="10"/>
       <c r="AA37" s="10"/>
     </row>
-    <row r="38" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="11" t="s">
         <v>221</v>
       </c>
@@ -22653,7 +22742,7 @@
       <c r="Z38" s="10"/>
       <c r="AA38" s="10"/>
     </row>
-    <row r="39" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
         <v>222</v>
       </c>
@@ -22690,7 +22779,7 @@
       <c r="Z39" s="10"/>
       <c r="AA39" s="10"/>
     </row>
-    <row r="40" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
         <v>223</v>
       </c>
@@ -22727,7 +22816,7 @@
       <c r="Z40" s="10"/>
       <c r="AA40" s="10"/>
     </row>
-    <row r="41" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="11" t="s">
         <v>224</v>
       </c>
@@ -22764,7 +22853,7 @@
       <c r="Z41" s="10"/>
       <c r="AA41" s="10"/>
     </row>
-    <row r="42" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="11" t="s">
         <v>225</v>
       </c>
@@ -22801,7 +22890,7 @@
       <c r="Z42" s="10"/>
       <c r="AA42" s="10"/>
     </row>
-    <row r="43" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="11" t="s">
         <v>226</v>
       </c>
@@ -22838,7 +22927,7 @@
       <c r="Z43" s="10"/>
       <c r="AA43" s="10"/>
     </row>
-    <row r="44" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="11" t="s">
         <v>227</v>
       </c>
@@ -22875,7 +22964,7 @@
       <c r="Z44" s="10"/>
       <c r="AA44" s="10"/>
     </row>
-    <row r="45" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="11" t="s">
         <v>228</v>
       </c>
@@ -22914,7 +23003,7 @@
       <c r="Z45" s="10"/>
       <c r="AA45" s="10"/>
     </row>
-    <row r="46" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="11" t="s">
         <v>229</v>
       </c>
@@ -22953,7 +23042,7 @@
       <c r="Z46" s="10"/>
       <c r="AA46" s="10"/>
     </row>
-    <row r="47" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
         <v>230</v>
       </c>
@@ -22992,7 +23081,7 @@
       <c r="Z47" s="10"/>
       <c r="AA47" s="10"/>
     </row>
-    <row r="48" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="11" t="s">
         <v>231</v>
       </c>
@@ -23031,7 +23120,7 @@
       <c r="Z48" s="10"/>
       <c r="AA48" s="10"/>
     </row>
-    <row r="49" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
         <v>232</v>
       </c>
@@ -23070,7 +23159,7 @@
       <c r="Z49" s="10"/>
       <c r="AA49" s="10"/>
     </row>
-    <row r="50" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="11" t="s">
         <v>233</v>
       </c>
@@ -23109,7 +23198,7 @@
       <c r="Z50" s="10"/>
       <c r="AA50" s="10"/>
     </row>
-    <row r="51" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="11" t="s">
         <v>234</v>
       </c>
@@ -23148,7 +23237,7 @@
       <c r="Z51" s="10"/>
       <c r="AA51" s="10"/>
     </row>
-    <row r="52" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="11" t="s">
         <v>235</v>
       </c>
@@ -23187,7 +23276,7 @@
       <c r="Z52" s="10"/>
       <c r="AA52" s="10"/>
     </row>
-    <row r="53" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="11" t="s">
         <v>236</v>
       </c>
@@ -23226,7 +23315,7 @@
       <c r="Z53" s="10"/>
       <c r="AA53" s="10"/>
     </row>
-    <row r="54" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="11" t="s">
         <v>237</v>
       </c>
@@ -23265,7 +23354,7 @@
       <c r="Z54" s="10"/>
       <c r="AA54" s="10"/>
     </row>
-    <row r="55" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="11" t="s">
         <v>238</v>
       </c>
@@ -23304,7 +23393,7 @@
       <c r="Z55" s="10"/>
       <c r="AA55" s="10"/>
     </row>
-    <row r="56" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="11" t="s">
         <v>239</v>
       </c>
@@ -23343,7 +23432,7 @@
       <c r="Z56" s="10"/>
       <c r="AA56" s="10"/>
     </row>
-    <row r="57" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="11" t="s">
         <v>240</v>
       </c>
@@ -23382,7 +23471,7 @@
       <c r="Z57" s="10"/>
       <c r="AA57" s="10"/>
     </row>
-    <row r="58" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="11" t="s">
         <v>241</v>
       </c>
@@ -23421,7 +23510,7 @@
       <c r="Z58" s="10"/>
       <c r="AA58" s="10"/>
     </row>
-    <row r="59" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="11" t="s">
         <v>242</v>
       </c>
@@ -23460,7 +23549,7 @@
       <c r="Z59" s="10"/>
       <c r="AA59" s="10"/>
     </row>
-    <row r="60" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="11" t="s">
         <v>243</v>
       </c>
@@ -23501,7 +23590,7 @@
       <c r="Z60" s="10"/>
       <c r="AA60" s="10"/>
     </row>
-    <row r="61" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="11" t="s">
         <v>244</v>
       </c>
@@ -23542,7 +23631,7 @@
       <c r="Z61" s="10"/>
       <c r="AA61" s="10"/>
     </row>
-    <row r="62" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="11" t="s">
         <v>245</v>
       </c>
@@ -23583,7 +23672,7 @@
       <c r="Z62" s="10"/>
       <c r="AA62" s="10"/>
     </row>
-    <row r="63" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="11" t="s">
         <v>246</v>
       </c>
@@ -23624,7 +23713,7 @@
       <c r="Z63" s="10"/>
       <c r="AA63" s="10"/>
     </row>
-    <row r="64" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="11" t="s">
         <v>247</v>
       </c>
@@ -23665,7 +23754,7 @@
       <c r="Z64" s="10"/>
       <c r="AA64" s="10"/>
     </row>
-    <row r="65" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="11" t="s">
         <v>248</v>
       </c>
@@ -23706,7 +23795,7 @@
       <c r="Z65" s="10"/>
       <c r="AA65" s="10"/>
     </row>
-    <row r="66" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="11" t="s">
         <v>249</v>
       </c>

</xml_diff>